<commit_message>
Acrescenta análise do Prelúdio BWV 558 com compassos reais
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XsRadmpgMkqHXAc1ma1Zn1
</commit_message>
<xml_diff>
--- a/grelhas-avaliacao-leonor-silva.xlsx
+++ b/grelhas-avaliacao-leonor-silva.xlsx
@@ -3383,7 +3383,7 @@
       <c r="AC51" s="13" t="n"/>
       <c r="AD51" s="13" t="inlineStr">
         <is>
-          <t>TESTE II (2.º sem.) – Mib M/dó m + Prelúdio + Pachelbel</t>
+          <t>TESTE II (2.º sem.) – Mib M/dó m + Prelúdio BWV 558 + Pachelbel</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="F2" s="24" t="inlineStr">
         <is>
-          <t>Mib M/dó m · Prelúdio · Pachelbel</t>
+          <t>Mib M/dó m · Prelúdio BWV 558 · Pachelbel</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6735,7 @@
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Prelúdio (sol m)</t>
+          <t>Prelúdio BWV 558 (sol m)</t>
         </is>
       </c>
       <c r="B11" s="25" t="inlineStr">
@@ -6744,21 +6744,21 @@
         </is>
       </c>
       <c r="C11" s="25" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D11" s="25" t="n">
+        <v>44</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="F11" s="25" t="inlineStr">
+        <is>
+          <t>54–60</t>
+        </is>
+      </c>
+      <c r="G11" s="25" t="n">
         <v>48</v>
-      </c>
-      <c r="E11" s="25" t="n">
-        <v>54</v>
-      </c>
-      <c r="F11" s="25" t="inlineStr">
-        <is>
-          <t>56–63</t>
-        </is>
-      </c>
-      <c r="G11" s="25" t="n">
-        <v>50</v>
       </c>
       <c r="H11" s="26" t="n"/>
       <c r="I11" s="26" t="n"/>

</xml_diff>